<commit_message>
Fixed the bug. Needed to create the annual_totals array in the init function to prevent the same memory being accessed.
</commit_message>
<xml_diff>
--- a/self_consumption_total_by_household.xlsx
+++ b/self_consumption_total_by_household.xlsx
@@ -456,19 +456,19 @@
         <v>105</v>
       </c>
       <c r="C2" t="n">
-        <v>1230.707551401869</v>
+        <v>888.413121495327</v>
       </c>
       <c r="D2" t="n">
-        <v>1786.167691588785</v>
+        <v>1689.176551401869</v>
       </c>
       <c r="E2" t="n">
-        <v>129.1503551401869</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>-449.1181073850468</v>
+        <v>-571.9716150560748</v>
       </c>
       <c r="G2" t="n">
-        <v>-10.93220637542057</v>
+        <v>-24.85295937598132</v>
       </c>
     </row>
     <row r="3">
@@ -479,19 +479,19 @@
         <v>107</v>
       </c>
       <c r="C3" t="n">
-        <v>2974.061857142857</v>
+        <v>2485.261428571428</v>
       </c>
       <c r="D3" t="n">
-        <v>629.0485714285714</v>
+        <v>496.4301428571429</v>
       </c>
       <c r="E3" t="n">
-        <v>200.0000000000001</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>-264.8647846857143</v>
+        <v>-455.6932003142857</v>
       </c>
       <c r="G3" t="n">
-        <v>76.17937497</v>
+        <v>54.89384681499998</v>
       </c>
     </row>
     <row r="4">
@@ -499,22 +499,22 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>108</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>5561.476000000001</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>270.017</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>199.9999999999999</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>-227.4960682</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>157.22553042</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -522,22 +522,22 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>4153.475714285714</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>554.9477142857141</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>199.9999999999999</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>-250.7845662285715</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>108.5974437528571</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -545,22 +545,22 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>112</v>
+        <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>4320.137124999999</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>1139.033</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>178.195</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>-304.18996155</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>94.36919807875</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -568,22 +568,22 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>118</v>
+        <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>1417.495</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>1826.054</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>121.008</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>-409.3834616</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>-6.683277449999988</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -591,22 +591,22 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>119</v>
+        <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>941.2194285714286</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>2957.789285714286</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>109.0048571428572</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>-498.4427897142857</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>-55.26522294214286</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -614,22 +614,22 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>122</v>
+        <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>2598.95</v>
+        <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>568.753</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>200.0000000000001</v>
+        <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>-256.3805867999999</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>67.92538799500001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -637,22 +637,22 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>123</v>
+        <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>4313.697999999999</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>328.8049999999999</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>-224.7095526</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>122.537823895</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -660,22 +660,22 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>125</v>
+        <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>1761.164</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>1225.4</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>173.297</v>
+        <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>-333.8397336</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>26.38739342</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -683,22 +683,22 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>126</v>
+        <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>3686.289545454546</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>797.5027272727273</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>196.4717272727273</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>-268.1303960181818</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>89.87910793227275</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -706,22 +706,22 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>127</v>
+        <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>3356.884</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>926.559</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>-283.0361854</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>77.332083</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -729,22 +729,22 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>475.6098181818183</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>4061.049090909091</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>95.46245454545453</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>-602.8118081636364</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>-94.6011794068182</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -752,22 +752,22 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>133</v>
+        <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>1299.358243243243</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>2146.756243243243</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>112.1352162162162</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>-445.3942091405405</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>-17.1232740504054</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -775,22 +775,22 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>137</v>
+        <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>2741.299315789474</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>1435.069421052632</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>113.667052631579</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>-403.4862625263157</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>35.14869116184211</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -798,22 +798,22 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>140</v>
+        <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>6075.134</v>
+        <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>460.352</v>
+        <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>200.0000000000001</v>
+        <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>-234.0689121999999</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>166.93439291</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -821,22 +821,22 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>145</v>
+        <v>0</v>
       </c>
       <c r="C18" t="n">
-        <v>1463.454</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>2868.563</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>188.527</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>-469.2532332</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>-27.296439835</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -844,22 +844,22 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>148</v>
+        <v>0</v>
       </c>
       <c r="C19" t="n">
-        <v>1631.475</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>2904.705</v>
+        <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>-397.9733634</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>-22.856362825</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -867,22 +867,22 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>151</v>
+        <v>0</v>
       </c>
       <c r="C20" t="n">
-        <v>2244.540235294118</v>
+        <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>1183.189705882353</v>
+        <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>187.6421176470588</v>
+        <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>-307.1255475882353</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>39.327300925</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -890,22 +890,22 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>154</v>
+        <v>0</v>
       </c>
       <c r="C21" t="n">
-        <v>3473.035</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>901.2670000000001</v>
+        <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>192.006</v>
+        <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>-271.0305438</v>
+        <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>81.27576216</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -913,22 +913,22 @@
         <v>20</v>
       </c>
       <c r="B22" t="n">
-        <v>155</v>
+        <v>0</v>
       </c>
       <c r="C22" t="n">
-        <v>4591.313</v>
+        <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>269.0829999999999</v>
+        <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>199.9999999999999</v>
+        <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>-231.5223876</v>
+        <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>132.24770989</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -936,22 +936,22 @@
         <v>21</v>
       </c>
       <c r="B23" t="n">
-        <v>156</v>
+        <v>0</v>
       </c>
       <c r="C23" t="n">
-        <v>1339.895</v>
+        <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>2174.088</v>
+        <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>122.081</v>
+        <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>-469.1915554</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>-17.74275242500001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -959,22 +959,22 @@
         <v>22</v>
       </c>
       <c r="B24" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="C24" t="n">
-        <v>4141.506</v>
+        <v>0</v>
       </c>
       <c r="D24" t="n">
-        <v>205.194</v>
+        <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>200.0000000000001</v>
+        <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>-239.8519731999999</v>
+        <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>120.96622846</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -982,22 +982,22 @@
         <v>23</v>
       </c>
       <c r="B25" t="n">
-        <v>160</v>
+        <v>0</v>
       </c>
       <c r="C25" t="n">
-        <v>1282.138073170732</v>
+        <v>0</v>
       </c>
       <c r="D25" t="n">
-        <v>2383.094585365853</v>
+        <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>153.3799756097561</v>
+        <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>-429.7331558341463</v>
+        <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>-20.39626908634146</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -1005,22 +1005,22 @@
         <v>24</v>
       </c>
       <c r="B26" t="n">
-        <v>161</v>
+        <v>0</v>
       </c>
       <c r="C26" t="n">
-        <v>2296.437125</v>
+        <v>0</v>
       </c>
       <c r="D26" t="n">
-        <v>3138.164</v>
+        <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>89.68175000000001</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>-539.74347005</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>-32.85754789999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -1028,22 +1028,22 @@
         <v>25</v>
       </c>
       <c r="B27" t="n">
-        <v>163</v>
+        <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>5802.167</v>
+        <v>0</v>
       </c>
       <c r="D27" t="n">
-        <v>105.3846279069767</v>
+        <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>-223.3142495581395</v>
+        <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>169.280993903721</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1051,22 +1051,22 @@
         <v>26</v>
       </c>
       <c r="B28" t="n">
-        <v>167</v>
+        <v>0</v>
       </c>
       <c r="C28" t="n">
-        <v>9626.967000000001</v>
+        <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>435.477</v>
+        <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>200.0000000000001</v>
+        <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>-232.1906439999999</v>
+        <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>262.975231135</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -1074,22 +1074,22 @@
         <v>27</v>
       </c>
       <c r="B29" t="n">
-        <v>168</v>
+        <v>0</v>
       </c>
       <c r="C29" t="n">
-        <v>5205.567818181818</v>
+        <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>200.3752727272728</v>
+        <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>-228.0605432909091</v>
+        <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>150.6306255813636</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -1097,22 +1097,22 @@
         <v>28</v>
       </c>
       <c r="B30" t="n">
-        <v>173</v>
+        <v>0</v>
       </c>
       <c r="C30" t="n">
-        <v>2424.810692307693</v>
+        <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>1695.882538461539</v>
+        <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>164.1985384615385</v>
+        <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>-387.0758026153846</v>
+        <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>27.061315765</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -1120,22 +1120,22 @@
         <v>29</v>
       </c>
       <c r="B31" t="n">
-        <v>174</v>
+        <v>0</v>
       </c>
       <c r="C31" t="n">
-        <v>3028.832780487804</v>
+        <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>1480.786975609756</v>
+        <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>140.3369024390244</v>
+        <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>-376.6998212390243</v>
+        <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>52.05824779170732</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -1143,22 +1143,22 @@
         <v>30</v>
       </c>
       <c r="B32" t="n">
-        <v>178</v>
+        <v>0</v>
       </c>
       <c r="C32" t="n">
-        <v>2900.128</v>
+        <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>319.3629999999999</v>
+        <v>0</v>
       </c>
       <c r="E32" t="n">
-        <v>192.505</v>
+        <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>-250.3649022</v>
+        <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>82.08128035499999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -1166,22 +1166,22 @@
         <v>31</v>
       </c>
       <c r="B33" t="n">
-        <v>184</v>
+        <v>0</v>
       </c>
       <c r="C33" t="n">
-        <v>5264.862</v>
+        <v>0</v>
       </c>
       <c r="D33" t="n">
-        <v>268.5382857142856</v>
+        <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>199.9999999999999</v>
+        <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>-232.2045551142858</v>
+        <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>149.5520947028571</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -1189,22 +1189,22 @@
         <v>32</v>
       </c>
       <c r="B34" t="n">
-        <v>186</v>
+        <v>0</v>
       </c>
       <c r="C34" t="n">
-        <v>4473.533341463415</v>
+        <v>0</v>
       </c>
       <c r="D34" t="n">
-        <v>179.0622926829267</v>
+        <v>0</v>
       </c>
       <c r="E34" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>-227.2026269609757</v>
+        <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>131.0184639578049</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -1212,22 +1212,22 @@
         <v>33</v>
       </c>
       <c r="B35" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="C35" t="n">
-        <v>1899.912571428571</v>
+        <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>2006.600238095238</v>
+        <v>0</v>
       </c>
       <c r="E35" t="n">
-        <v>132.224</v>
+        <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>-413.7021990952381</v>
+        <v>0</v>
       </c>
       <c r="G35" t="n">
-        <v>1.12206982333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -1235,22 +1235,22 @@
         <v>34</v>
       </c>
       <c r="B36" t="n">
-        <v>193</v>
+        <v>0</v>
       </c>
       <c r="C36" t="n">
-        <v>1086.726</v>
+        <v>0</v>
       </c>
       <c r="D36" t="n">
-        <v>2340.2895</v>
+        <v>0</v>
       </c>
       <c r="E36" t="n">
-        <v>110.4725</v>
+        <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>-477.112419</v>
+        <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>-29.2706569525</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -1258,22 +1258,22 @@
         <v>35</v>
       </c>
       <c r="B37" t="n">
-        <v>194</v>
+        <v>0</v>
       </c>
       <c r="C37" t="n">
-        <v>3274.812</v>
+        <v>0</v>
       </c>
       <c r="D37" t="n">
-        <v>1904.538</v>
+        <v>0</v>
       </c>
       <c r="E37" t="n">
-        <v>121.826</v>
+        <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>-437.9345798000001</v>
+        <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>39.75936982500001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -1281,22 +1281,22 @@
         <v>36</v>
       </c>
       <c r="B38" t="n">
-        <v>196</v>
+        <v>0</v>
       </c>
       <c r="C38" t="n">
-        <v>2256.18</v>
+        <v>0</v>
       </c>
       <c r="D38" t="n">
-        <v>2113.213</v>
+        <v>0</v>
       </c>
       <c r="E38" t="n">
-        <v>128.439</v>
+        <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>-416.0106598</v>
+        <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>9.186221445000005</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -1304,22 +1304,22 @@
         <v>37</v>
       </c>
       <c r="B39" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="C39" t="n">
-        <v>6702.509000000001</v>
+        <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v>38.96142857142858</v>
+        <v>0</v>
       </c>
       <c r="E39" t="n">
-        <v>199.9999999999999</v>
+        <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>-208.5410672857143</v>
+        <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>199.5074330428571</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -1327,22 +1327,22 @@
         <v>38</v>
       </c>
       <c r="B40" t="n">
-        <v>202</v>
+        <v>0</v>
       </c>
       <c r="C40" t="n">
-        <v>5762.997857142856</v>
+        <v>0</v>
       </c>
       <c r="D40" t="n">
-        <v>333.3342857142857</v>
+        <v>0</v>
       </c>
       <c r="E40" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>-230.7011713428572</v>
+        <v>0</v>
       </c>
       <c r="G40" t="n">
-        <v>161.48316401</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -1350,22 +1350,22 @@
         <v>39</v>
       </c>
       <c r="B41" t="n">
-        <v>204</v>
+        <v>0</v>
       </c>
       <c r="C41" t="n">
-        <v>2905.041278481012</v>
+        <v>0</v>
       </c>
       <c r="D41" t="n">
-        <v>388.7527974683545</v>
+        <v>0</v>
       </c>
       <c r="E41" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>-241.6186745898734</v>
+        <v>0</v>
       </c>
       <c r="G41" t="n">
-        <v>82.09328630689873</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -1373,22 +1373,22 @@
         <v>40</v>
       </c>
       <c r="B42" t="n">
-        <v>206</v>
+        <v>0</v>
       </c>
       <c r="C42" t="n">
-        <v>2059.419842105263</v>
+        <v>0</v>
       </c>
       <c r="D42" t="n">
-        <v>2392.590999999999</v>
+        <v>0</v>
       </c>
       <c r="E42" t="n">
-        <v>186.0162105263158</v>
+        <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>-394.7101683578947</v>
+        <v>0</v>
       </c>
       <c r="G42" t="n">
-        <v>0.2983732721052661</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -1396,22 +1396,22 @@
         <v>41</v>
       </c>
       <c r="B43" t="n">
-        <v>208</v>
+        <v>0</v>
       </c>
       <c r="C43" t="n">
-        <v>3718.194</v>
+        <v>0</v>
       </c>
       <c r="D43" t="n">
-        <v>697.4691666666665</v>
+        <v>0</v>
       </c>
       <c r="E43" t="n">
-        <v>195.7503333333333</v>
+        <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>-252.4581015666667</v>
+        <v>0</v>
       </c>
       <c r="G43" t="n">
-        <v>95.42534529333334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -1419,22 +1419,22 @@
         <v>42</v>
       </c>
       <c r="B44" t="n">
-        <v>209</v>
+        <v>0</v>
       </c>
       <c r="C44" t="n">
-        <v>2019.471</v>
+        <v>0</v>
       </c>
       <c r="D44" t="n">
-        <v>1312.497</v>
+        <v>0</v>
       </c>
       <c r="E44" t="n">
-        <v>136.884</v>
+        <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>-368.0143482</v>
+        <v>0</v>
       </c>
       <c r="G44" t="n">
-        <v>23.86777762500001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -1442,22 +1442,22 @@
         <v>43</v>
       </c>
       <c r="B45" t="n">
-        <v>210</v>
+        <v>0</v>
       </c>
       <c r="C45" t="n">
-        <v>3800.475615384616</v>
+        <v>0</v>
       </c>
       <c r="D45" t="n">
-        <v>1051.281538461538</v>
+        <v>0</v>
       </c>
       <c r="E45" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>-267.0021021384615</v>
+        <v>0</v>
       </c>
       <c r="G45" t="n">
-        <v>86.98648093153847</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -1465,22 +1465,22 @@
         <v>44</v>
       </c>
       <c r="B46" t="n">
-        <v>212</v>
+        <v>0</v>
       </c>
       <c r="C46" t="n">
-        <v>1258.225142857143</v>
+        <v>0</v>
       </c>
       <c r="D46" t="n">
-        <v>2880.262714285715</v>
+        <v>0</v>
       </c>
       <c r="E46" t="n">
-        <v>146.114</v>
+        <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>-457.6347533714286</v>
+        <v>0</v>
       </c>
       <c r="G46" t="n">
-        <v>-39.92112737642857</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1488,22 +1488,22 @@
         <v>45</v>
       </c>
       <c r="B47" t="n">
-        <v>215</v>
+        <v>0</v>
       </c>
       <c r="C47" t="n">
-        <v>3475.792</v>
+        <v>0</v>
       </c>
       <c r="D47" t="n">
-        <v>3404.554</v>
+        <v>0</v>
       </c>
       <c r="E47" t="n">
-        <v>138.591</v>
+        <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>-477.1362494</v>
+        <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>6.401591049999986</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -1511,22 +1511,22 @@
         <v>46</v>
       </c>
       <c r="B48" t="n">
-        <v>217</v>
+        <v>0</v>
       </c>
       <c r="C48" t="n">
-        <v>1796.507454545454</v>
+        <v>0</v>
       </c>
       <c r="D48" t="n">
-        <v>2071.323181818182</v>
+        <v>0</v>
       </c>
       <c r="E48" t="n">
-        <v>124.0972727272727</v>
+        <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>-443.4246284000001</v>
+        <v>0</v>
       </c>
       <c r="G48" t="n">
-        <v>-4.423001271363638</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -1534,22 +1534,22 @@
         <v>47</v>
       </c>
       <c r="B49" t="n">
-        <v>219</v>
+        <v>0</v>
       </c>
       <c r="C49" t="n">
-        <v>4622.906463414634</v>
+        <v>0</v>
       </c>
       <c r="D49" t="n">
-        <v>215.9133658536585</v>
+        <v>0</v>
       </c>
       <c r="E49" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>-230.0627086243902</v>
+        <v>0</v>
       </c>
       <c r="G49" t="n">
-        <v>132.9859366965854</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -1557,22 +1557,22 @@
         <v>48</v>
       </c>
       <c r="B50" t="n">
-        <v>223</v>
+        <v>0</v>
       </c>
       <c r="C50" t="n">
-        <v>3585.665999999999</v>
+        <v>0</v>
       </c>
       <c r="D50" t="n">
-        <v>1122.494823529412</v>
+        <v>0</v>
       </c>
       <c r="E50" t="n">
-        <v>158.9025294117647</v>
+        <v>0</v>
       </c>
       <c r="F50" t="n">
-        <v>-340.2652499176471</v>
+        <v>0</v>
       </c>
       <c r="G50" t="n">
-        <v>72.82163459676468</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -1580,22 +1580,22 @@
         <v>49</v>
       </c>
       <c r="B51" t="n">
-        <v>225</v>
+        <v>0</v>
       </c>
       <c r="C51" t="n">
-        <v>1998.587727272728</v>
+        <v>0</v>
       </c>
       <c r="D51" t="n">
-        <v>1653.008454545455</v>
+        <v>0</v>
       </c>
       <c r="E51" t="n">
-        <v>132.4905454545454</v>
+        <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>-394.3038188</v>
+        <v>0</v>
       </c>
       <c r="G51" t="n">
-        <v>12.73943626</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -1603,22 +1603,22 @@
         <v>50</v>
       </c>
       <c r="B52" t="n">
-        <v>226</v>
+        <v>0</v>
       </c>
       <c r="C52" t="n">
-        <v>4038.893548387098</v>
+        <v>0</v>
       </c>
       <c r="D52" t="n">
-        <v>578.0743870967742</v>
+        <v>0</v>
       </c>
       <c r="E52" t="n">
-        <v>189.6605483870968</v>
+        <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>-269.6099800774194</v>
+        <v>0</v>
       </c>
       <c r="G52" t="n">
-        <v>103.9055188909678</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -1626,22 +1626,22 @@
         <v>51</v>
       </c>
       <c r="B53" t="n">
-        <v>227</v>
+        <v>0</v>
       </c>
       <c r="C53" t="n">
-        <v>3567.596</v>
+        <v>0</v>
       </c>
       <c r="D53" t="n">
-        <v>705.157</v>
+        <v>0</v>
       </c>
       <c r="E53" t="n">
-        <v>174.017</v>
+        <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>-283.7831162</v>
+        <v>0</v>
       </c>
       <c r="G53" t="n">
-        <v>86.834868895</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -1649,22 +1649,22 @@
         <v>52</v>
       </c>
       <c r="B54" t="n">
-        <v>232</v>
+        <v>0</v>
       </c>
       <c r="C54" t="n">
-        <v>601.8450000000003</v>
+        <v>0</v>
       </c>
       <c r="D54" t="n">
-        <v>4056.395272727273</v>
+        <v>0</v>
       </c>
       <c r="E54" t="n">
-        <v>98.43390909090907</v>
+        <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>-564.9645747272727</v>
+        <v>0</v>
       </c>
       <c r="G54" t="n">
-        <v>-98.73632526</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -1672,22 +1672,22 @@
         <v>53</v>
       </c>
       <c r="B55" t="n">
-        <v>235</v>
+        <v>0</v>
       </c>
       <c r="C55" t="n">
-        <v>4549.494</v>
+        <v>0</v>
       </c>
       <c r="D55" t="n">
-        <v>512.035</v>
+        <v>0</v>
       </c>
       <c r="E55" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F55" t="n">
-        <v>-258.4691508</v>
+        <v>0</v>
       </c>
       <c r="G55" t="n">
-        <v>121.25575163</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -1695,22 +1695,22 @@
         <v>54</v>
       </c>
       <c r="B56" t="n">
-        <v>239</v>
+        <v>0</v>
       </c>
       <c r="C56" t="n">
-        <v>4077.274</v>
+        <v>0</v>
       </c>
       <c r="D56" t="n">
-        <v>671.396</v>
+        <v>0</v>
       </c>
       <c r="E56" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>-247.2832564</v>
+        <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>108.71245356</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -1718,22 +1718,22 @@
         <v>55</v>
       </c>
       <c r="B57" t="n">
-        <v>241</v>
+        <v>0</v>
       </c>
       <c r="C57" t="n">
-        <v>5782.763000000001</v>
+        <v>0</v>
       </c>
       <c r="D57" t="n">
-        <v>368.917</v>
+        <v>0</v>
       </c>
       <c r="E57" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F57" t="n">
-        <v>-220.4027152</v>
+        <v>0</v>
       </c>
       <c r="G57" t="n">
-        <v>159.983842735</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -1741,22 +1741,22 @@
         <v>56</v>
       </c>
       <c r="B58" t="n">
-        <v>243</v>
+        <v>0</v>
       </c>
       <c r="C58" t="n">
-        <v>1599.377064516129</v>
+        <v>0</v>
       </c>
       <c r="D58" t="n">
-        <v>1941.044290322581</v>
+        <v>0</v>
       </c>
       <c r="E58" t="n">
-        <v>157.8538387096774</v>
+        <v>0</v>
       </c>
       <c r="F58" t="n">
-        <v>-401.9172362774194</v>
+        <v>0</v>
       </c>
       <c r="G58" t="n">
-        <v>-0.5477519688709735</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -1764,22 +1764,22 @@
         <v>57</v>
       </c>
       <c r="B59" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="C59" t="n">
-        <v>5358.534714285714</v>
+        <v>0</v>
       </c>
       <c r="D59" t="n">
-        <v>276.5634285714286</v>
+        <v>0</v>
       </c>
       <c r="E59" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F59" t="n">
-        <v>-233.9048250571428</v>
+        <v>0</v>
       </c>
       <c r="G59" t="n">
-        <v>151.2678286664286</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -1787,22 +1787,22 @@
         <v>58</v>
       </c>
       <c r="B60" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="C60" t="n">
-        <v>1166.209714285714</v>
+        <v>0</v>
       </c>
       <c r="D60" t="n">
-        <v>3144.998285714286</v>
+        <v>0</v>
       </c>
       <c r="E60" t="n">
-        <v>128.7565714285714</v>
+        <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>-509.9689202285715</v>
+        <v>0</v>
       </c>
       <c r="G60" t="n">
-        <v>-50.40150993214286</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -1810,22 +1810,22 @@
         <v>59</v>
       </c>
       <c r="B61" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="C61" t="n">
-        <v>2635.918</v>
+        <v>0</v>
       </c>
       <c r="D61" t="n">
-        <v>1079.779</v>
+        <v>0</v>
       </c>
       <c r="E61" t="n">
-        <v>171.029</v>
+        <v>0</v>
       </c>
       <c r="F61" t="n">
-        <v>-307.7479681999999</v>
+        <v>0</v>
       </c>
       <c r="G61" t="n">
-        <v>51.86042006000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -1833,22 +1833,22 @@
         <v>60</v>
       </c>
       <c r="B62" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="C62" t="n">
-        <v>3515.004857142857</v>
+        <v>0</v>
       </c>
       <c r="D62" t="n">
-        <v>827.6294285714289</v>
+        <v>0</v>
       </c>
       <c r="E62" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>-250.9442479428571</v>
+        <v>0</v>
       </c>
       <c r="G62" t="n">
-        <v>84.71107449142858</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63">
@@ -1856,22 +1856,22 @@
         <v>61</v>
       </c>
       <c r="B63" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="C63" t="n">
-        <v>1681.005333333334</v>
+        <v>0</v>
       </c>
       <c r="D63" t="n">
-        <v>2106.931</v>
+        <v>0</v>
       </c>
       <c r="E63" t="n">
-        <v>111.2866666666667</v>
+        <v>0</v>
       </c>
       <c r="F63" t="n">
-        <v>-466.2920312</v>
+        <v>0</v>
       </c>
       <c r="G63" t="n">
-        <v>-10.78016374166667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -1879,22 +1879,22 @@
         <v>62</v>
       </c>
       <c r="B64" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="C64" t="n">
-        <v>1967.385482758621</v>
+        <v>0</v>
       </c>
       <c r="D64" t="n">
-        <v>1016.189103448276</v>
+        <v>0</v>
       </c>
       <c r="E64" t="n">
-        <v>141.978</v>
+        <v>0</v>
       </c>
       <c r="F64" t="n">
-        <v>-362.8540889034483</v>
+        <v>0</v>
       </c>
       <c r="G64" t="n">
-        <v>32.52411541913793</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -1902,22 +1902,22 @@
         <v>63</v>
       </c>
       <c r="B65" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="C65" t="n">
-        <v>4441.294</v>
+        <v>0</v>
       </c>
       <c r="D65" t="n">
-        <v>369.5169999999999</v>
+        <v>0</v>
       </c>
       <c r="E65" t="n">
-        <v>199.9999999999999</v>
+        <v>0</v>
       </c>
       <c r="F65" t="n">
-        <v>-233.1868464</v>
+        <v>0</v>
       </c>
       <c r="G65" t="n">
-        <v>124.655502365</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
@@ -1925,22 +1925,22 @@
         <v>64</v>
       </c>
       <c r="B66" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="C66" t="n">
-        <v>2981.021838709677</v>
+        <v>0</v>
       </c>
       <c r="D66" t="n">
-        <v>997.2458064516131</v>
+        <v>0</v>
       </c>
       <c r="E66" t="n">
-        <v>166.0526129032257</v>
+        <v>0</v>
       </c>
       <c r="F66" t="n">
-        <v>-325.2194929354839</v>
+        <v>0</v>
       </c>
       <c r="G66" t="n">
-        <v>61.24164030209676</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67">
@@ -1948,22 +1948,22 @@
         <v>65</v>
       </c>
       <c r="B67" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="C67" t="n">
-        <v>2974.322</v>
+        <v>0</v>
       </c>
       <c r="D67" t="n">
-        <v>1294.886</v>
+        <v>0</v>
       </c>
       <c r="E67" t="n">
-        <v>183.331</v>
+        <v>0</v>
       </c>
       <c r="F67" t="n">
-        <v>-313.2582802</v>
+        <v>0</v>
       </c>
       <c r="G67" t="n">
-        <v>55.68894581999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
@@ -1971,22 +1971,22 @@
         <v>66</v>
       </c>
       <c r="B68" t="n">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="C68" t="n">
-        <v>2496.569707317073</v>
+        <v>0</v>
       </c>
       <c r="D68" t="n">
-        <v>1274.956414634146</v>
+        <v>0</v>
       </c>
       <c r="E68" t="n">
-        <v>172.9706829268293</v>
+        <v>0</v>
       </c>
       <c r="F68" t="n">
-        <v>-351.4223813609756</v>
+        <v>0</v>
       </c>
       <c r="G68" t="n">
-        <v>37.40747733756098</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
@@ -1994,22 +1994,22 @@
         <v>67</v>
       </c>
       <c r="B69" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="C69" t="n">
-        <v>195.9835714285715</v>
+        <v>0</v>
       </c>
       <c r="D69" t="n">
-        <v>5169.812</v>
+        <v>0</v>
       </c>
       <c r="E69" t="n">
-        <v>80.78228571428571</v>
+        <v>0</v>
       </c>
       <c r="F69" t="n">
-        <v>-668.0769296285714</v>
+        <v>0</v>
       </c>
       <c r="G69" t="n">
-        <v>-135.1998532792857</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70">
@@ -2017,22 +2017,22 @@
         <v>68</v>
       </c>
       <c r="B70" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="C70" t="n">
-        <v>3134.770428571429</v>
+        <v>0</v>
       </c>
       <c r="D70" t="n">
-        <v>1553.839714285714</v>
+        <v>0</v>
       </c>
       <c r="E70" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F70" t="n">
-        <v>-331.319078</v>
+        <v>0</v>
       </c>
       <c r="G70" t="n">
-        <v>54.35314884500001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -2040,22 +2040,22 @@
         <v>69</v>
       </c>
       <c r="B71" t="n">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="C71" t="n">
-        <v>1732.933</v>
+        <v>0</v>
       </c>
       <c r="D71" t="n">
-        <v>1468.564</v>
+        <v>0</v>
       </c>
       <c r="E71" t="n">
-        <v>132.814</v>
+        <v>0</v>
       </c>
       <c r="F71" t="n">
-        <v>-388.5764544</v>
+        <v>0</v>
       </c>
       <c r="G71" t="n">
-        <v>13.480072765</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -2063,22 +2063,22 @@
         <v>70</v>
       </c>
       <c r="B72" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="C72" t="n">
-        <v>2106.668</v>
+        <v>0</v>
       </c>
       <c r="D72" t="n">
-        <v>2487.752</v>
+        <v>0</v>
       </c>
       <c r="E72" t="n">
-        <v>135.34</v>
+        <v>0</v>
       </c>
       <c r="F72" t="n">
-        <v>-430.0386834</v>
+        <v>0</v>
       </c>
       <c r="G72" t="n">
-        <v>-5.296864604999996</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -2086,22 +2086,22 @@
         <v>71</v>
       </c>
       <c r="B73" t="n">
-        <v>66</v>
+        <v>0</v>
       </c>
       <c r="C73" t="n">
-        <v>3845.160749999999</v>
+        <v>0</v>
       </c>
       <c r="D73" t="n">
-        <v>546.9774999999998</v>
+        <v>0</v>
       </c>
       <c r="E73" t="n">
-        <v>164.46625</v>
+        <v>0</v>
       </c>
       <c r="F73" t="n">
-        <v>-284.35047845</v>
+        <v>0</v>
       </c>
       <c r="G73" t="n">
-        <v>99.05622592249998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -2109,22 +2109,22 @@
         <v>72</v>
       </c>
       <c r="B74" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="C74" t="n">
-        <v>2385.5</v>
+        <v>0</v>
       </c>
       <c r="D74" t="n">
-        <v>641.7699999999999</v>
+        <v>0</v>
       </c>
       <c r="E74" t="n">
-        <v>200.0000000000001</v>
+        <v>0</v>
       </c>
       <c r="F74" t="n">
-        <v>-262.5780894</v>
+        <v>0</v>
       </c>
       <c r="G74" t="n">
-        <v>63.00022454</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -2132,22 +2132,22 @@
         <v>73</v>
       </c>
       <c r="B75" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="C75" t="n">
-        <v>1360.004487804878</v>
+        <v>0</v>
       </c>
       <c r="D75" t="n">
-        <v>1201.578463414634</v>
+        <v>0</v>
       </c>
       <c r="E75" t="n">
-        <v>168.7719512195122</v>
+        <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>-332.3988607170731</v>
+        <v>0</v>
       </c>
       <c r="G75" t="n">
-        <v>15.42358298963415</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -2155,22 +2155,22 @@
         <v>74</v>
       </c>
       <c r="B76" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="C76" t="n">
-        <v>756.1130000000001</v>
+        <v>0</v>
       </c>
       <c r="D76" t="n">
-        <v>2968.531</v>
+        <v>0</v>
       </c>
       <c r="E76" t="n">
-        <v>123.088</v>
+        <v>0</v>
       </c>
       <c r="F76" t="n">
-        <v>-488.2148188</v>
+        <v>0</v>
       </c>
       <c r="G76" t="n">
-        <v>-53.87138505</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77">
@@ -2178,22 +2178,22 @@
         <v>75</v>
       </c>
       <c r="B77" t="n">
-        <v>71</v>
+        <v>0</v>
       </c>
       <c r="C77" t="n">
-        <v>1532.566</v>
+        <v>0</v>
       </c>
       <c r="D77" t="n">
-        <v>1631.446</v>
+        <v>0</v>
       </c>
       <c r="E77" t="n">
-        <v>139.735</v>
+        <v>0</v>
       </c>
       <c r="F77" t="n">
-        <v>-375.3495758</v>
+        <v>0</v>
       </c>
       <c r="G77" t="n">
-        <v>3.392014864999993</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78">
@@ -2201,22 +2201,22 @@
         <v>76</v>
       </c>
       <c r="B78" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="C78" t="n">
-        <v>4423.349</v>
+        <v>0</v>
       </c>
       <c r="D78" t="n">
-        <v>377.7340000000001</v>
+        <v>0</v>
       </c>
       <c r="E78" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F78" t="n">
-        <v>-239.222084</v>
+        <v>0</v>
       </c>
       <c r="G78" t="n">
-        <v>124.63834759</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -2224,22 +2224,22 @@
         <v>77</v>
       </c>
       <c r="B79" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="C79" t="n">
-        <v>1588.5075</v>
+        <v>0</v>
       </c>
       <c r="D79" t="n">
-        <v>2096.50725</v>
+        <v>0</v>
       </c>
       <c r="E79" t="n">
-        <v>200.0000000000001</v>
+        <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>-354.9831849999999</v>
+        <v>0</v>
       </c>
       <c r="G79" t="n">
-        <v>0.738844041250001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
@@ -2247,22 +2247,22 @@
         <v>78</v>
       </c>
       <c r="B80" t="n">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="C80" t="n">
-        <v>4551.757073170732</v>
+        <v>0</v>
       </c>
       <c r="D80" t="n">
-        <v>612.4002195121949</v>
+        <v>0</v>
       </c>
       <c r="E80" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F80" t="n">
-        <v>-257.4260569560976</v>
+        <v>0</v>
       </c>
       <c r="G80" t="n">
-        <v>118.6411453514634</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
@@ -2270,22 +2270,22 @@
         <v>79</v>
       </c>
       <c r="B81" t="n">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="C81" t="n">
-        <v>2711.654441558441</v>
+        <v>0</v>
       </c>
       <c r="D81" t="n">
-        <v>413.1205194805195</v>
+        <v>0</v>
       </c>
       <c r="E81" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F81" t="n">
-        <v>-241.8854800051948</v>
+        <v>0</v>
       </c>
       <c r="G81" t="n">
-        <v>79.47459500220776</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82">
@@ -2293,22 +2293,22 @@
         <v>80</v>
       </c>
       <c r="B82" t="n">
-        <v>84</v>
+        <v>0</v>
       </c>
       <c r="C82" t="n">
-        <v>567.2611428571428</v>
+        <v>0</v>
       </c>
       <c r="D82" t="n">
-        <v>3433.529285714285</v>
+        <v>0</v>
       </c>
       <c r="E82" t="n">
-        <v>126.9858571428572</v>
+        <v>0</v>
       </c>
       <c r="F82" t="n">
-        <v>-500.0692402571428</v>
+        <v>0</v>
       </c>
       <c r="G82" t="n">
-        <v>-71.02349143714285</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -2316,22 +2316,22 @@
         <v>81</v>
       </c>
       <c r="B83" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="C83" t="n">
-        <v>5675.974</v>
+        <v>0</v>
       </c>
       <c r="D83" t="n">
-        <v>54.947</v>
+        <v>0</v>
       </c>
       <c r="E83" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F83" t="n">
-        <v>-216.9830105999999</v>
+        <v>0</v>
       </c>
       <c r="G83" t="n">
-        <v>169.505844715</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84">
@@ -2339,22 +2339,22 @@
         <v>82</v>
       </c>
       <c r="B84" t="n">
-        <v>88</v>
+        <v>0</v>
       </c>
       <c r="C84" t="n">
-        <v>7010.878000000001</v>
+        <v>0</v>
       </c>
       <c r="D84" t="n">
-        <v>81.89900000000002</v>
+        <v>0</v>
       </c>
       <c r="E84" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F84" t="n">
-        <v>-216.9655836</v>
+        <v>0</v>
       </c>
       <c r="G84" t="n">
-        <v>205.6460204633333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
@@ -2362,22 +2362,22 @@
         <v>83</v>
       </c>
       <c r="B85" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="C85" t="n">
-        <v>1567.869</v>
+        <v>0</v>
       </c>
       <c r="D85" t="n">
-        <v>3027.379571428571</v>
+        <v>0</v>
       </c>
       <c r="E85" t="n">
-        <v>190.2984285714286</v>
+        <v>0</v>
       </c>
       <c r="F85" t="n">
-        <v>-410.5721419714286</v>
+        <v>0</v>
       </c>
       <c r="G85" t="n">
-        <v>-27.7492132192857</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -2385,22 +2385,22 @@
         <v>84</v>
       </c>
       <c r="B86" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="C86" t="n">
-        <v>464.081</v>
+        <v>0</v>
       </c>
       <c r="D86" t="n">
-        <v>8284.849000000002</v>
+        <v>0</v>
       </c>
       <c r="E86" t="n">
-        <v>55.20100000000001</v>
+        <v>0</v>
       </c>
       <c r="F86" t="n">
-        <v>-1028.8543372</v>
+        <v>0</v>
       </c>
       <c r="G86" t="n">
-        <v>-238.260670055</v>
+        <v>0</v>
       </c>
     </row>
     <row r="87">
@@ -2408,22 +2408,22 @@
         <v>85</v>
       </c>
       <c r="B87" t="n">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="C87" t="n">
-        <v>627.1940000000001</v>
+        <v>0</v>
       </c>
       <c r="D87" t="n">
-        <v>1688.623</v>
+        <v>0</v>
       </c>
       <c r="E87" t="n">
-        <v>112.201</v>
+        <v>0</v>
       </c>
       <c r="F87" t="n">
-        <v>-406.399207</v>
+        <v>0</v>
       </c>
       <c r="G87" t="n">
-        <v>-23.122474925</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -2431,22 +2431,22 @@
         <v>86</v>
       </c>
       <c r="B88" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="C88" t="n">
-        <v>1919.007</v>
+        <v>0</v>
       </c>
       <c r="D88" t="n">
-        <v>649.673</v>
+        <v>0</v>
       </c>
       <c r="E88" t="n">
-        <v>197.857</v>
+        <v>0</v>
       </c>
       <c r="F88" t="n">
-        <v>-257.2100798</v>
+        <v>0</v>
       </c>
       <c r="G88" t="n">
-        <v>47.35206222500001</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final commit before seminar.
</commit_message>
<xml_diff>
--- a/self_consumption_total_by_household.xlsx
+++ b/self_consumption_total_by_household.xlsx
@@ -499,22 +499,22 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>108</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>5006.166999999999</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>166.668</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>-418.1282858</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>134.790424855</v>
       </c>
     </row>
     <row r="5">
@@ -522,22 +522,22 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>3562.196142857144</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>395.1515714285713</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>-436.6269722857143</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>87.57098383642858</v>
       </c>
     </row>
     <row r="6">
@@ -545,22 +545,22 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>112</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>3887.440500000001</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1075.699375</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>-478.30706795</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>77.135183511875</v>
       </c>
     </row>
     <row r="7">
@@ -568,22 +568,22 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>1074.388</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>1729.259</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>-524.992488</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>-20.36512335</v>
       </c>
     </row>
     <row r="8">
@@ -591,22 +591,22 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>119</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>660.7091428571428</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>2853.234142857143</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>-600.6465049428572</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>-66.27813899357145</v>
       </c>
     </row>
     <row r="9">
@@ -614,22 +614,22 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>122</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>2106.527</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>437.148</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>-447.1302969999999</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>47.26157906499999</v>
       </c>
     </row>
     <row r="10">
@@ -637,22 +637,22 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>123</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>3758.332</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>236.07</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>-416.6260238</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>99.77086012500001</v>
       </c>
     </row>
     <row r="11">
@@ -660,22 +660,22 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>1322.162</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>1063.704</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>-496.4407472</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>7.87318599</v>
       </c>
     </row>
     <row r="12">
@@ -683,22 +683,22 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>126</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>3053.84618181818</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>642.7975454545456</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>-453.5119925636363</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>66.13951402318179</v>
       </c>
     </row>
     <row r="13">
@@ -706,22 +706,22 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>127</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>2875.726</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>804.819</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>-474.118308</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>57.10787218499999</v>
       </c>
     </row>
     <row r="14">
@@ -729,22 +729,22 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>129</v>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>279.4109999999998</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>3969.198090909092</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>-691.7140268000001</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>-102.8896505986364</v>
       </c>
     </row>
     <row r="15">
@@ -752,22 +752,22 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>133</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>1038.308810810811</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>2061.053405405405</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>-552.6221581513513</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>-28.2506374072973</v>
       </c>
     </row>
     <row r="16">
@@ -775,22 +775,22 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>137</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>2355.940894736843</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>1365.253315789474</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>-513.8388630105263</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>21.05027640578948</v>
       </c>
     </row>
     <row r="17">
@@ -798,22 +798,22 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>5676.065000000001</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>366.563</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>-422.9655724</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>147.909051925</v>
       </c>
     </row>
     <row r="18">
@@ -821,22 +821,22 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>1005.504</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>2719.712</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>-648.0603547999999</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>-45.95595656499999</v>
       </c>
     </row>
     <row r="19">
@@ -844,22 +844,22 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>0</v>
+        <v>148</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>1270.147</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>2772.891</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>-585.7501517999999</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>-41.487806345</v>
       </c>
     </row>
     <row r="20">
@@ -867,22 +867,22 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>0</v>
+        <v>151</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>1782.757058823529</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1041.732294117647</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>-485.2297096</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>20.63079232558823</v>
       </c>
     </row>
     <row r="21">
@@ -890,22 +890,22 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>154</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>2938.804</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>798.096</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>-454.2971294</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>60.15991452</v>
       </c>
     </row>
     <row r="22">
@@ -913,22 +913,22 @@
         <v>20</v>
       </c>
       <c r="B22" t="n">
-        <v>0</v>
+        <v>155</v>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>4105.754</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>173.974</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>-421.43681</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>111.556988045</v>
       </c>
     </row>
     <row r="23">
@@ -936,22 +936,22 @@
         <v>21</v>
       </c>
       <c r="B23" t="n">
-        <v>0</v>
+        <v>156</v>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>1038.874</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>2077.459</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>-585.3272094</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>-30.73935407</v>
       </c>
     </row>
     <row r="24">
@@ -959,22 +959,22 @@
         <v>22</v>
       </c>
       <c r="B24" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
+        <v>3596.346</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>108.67</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>-430.4156348</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>98.321993015</v>
       </c>
     </row>
     <row r="25">
@@ -982,22 +982,22 @@
         <v>23</v>
       </c>
       <c r="B25" t="n">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>930.3228536585372</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>2236.939365853658</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>-572.2253477658536</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>-34.92904743902436</v>
       </c>
     </row>
     <row r="26">
@@ -1005,22 +1005,22 @@
         <v>24</v>
       </c>
       <c r="B26" t="n">
-        <v>0</v>
+        <v>161</v>
       </c>
       <c r="C26" t="n">
-        <v>0</v>
+        <v>1995.545125</v>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>3078.4305</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>0</v>
+        <v>-627.334185775</v>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>-43.72333088687503</v>
       </c>
     </row>
     <row r="27">
@@ -1028,22 +1028,22 @@
         <v>25</v>
       </c>
       <c r="B27" t="n">
-        <v>0</v>
+        <v>163</v>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>5324.016162790698</v>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>43.14537209302327</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>-417.5357594930232</v>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>147.4576220444186</v>
       </c>
     </row>
     <row r="28">
@@ -1051,22 +1051,22 @@
         <v>26</v>
       </c>
       <c r="B28" t="n">
-        <v>0</v>
+        <v>167</v>
       </c>
       <c r="C28" t="n">
-        <v>0</v>
+        <v>8746.575000000001</v>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>330.467</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>-422.6392396</v>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
+        <v>234.93169202</v>
       </c>
     </row>
     <row r="29">
@@ -1074,22 +1074,22 @@
         <v>27</v>
       </c>
       <c r="B29" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>4576.834727272727</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>99.17672727272733</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>-417.0956798363636</v>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>125.7993865863636</v>
       </c>
     </row>
     <row r="30">
@@ -1097,22 +1097,22 @@
         <v>28</v>
       </c>
       <c r="B30" t="n">
-        <v>0</v>
+        <v>173</v>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>1929.182692307692</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>1558.834076923077</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>0</v>
+        <v>-540.3627144615384</v>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>8.014695885769219</v>
       </c>
     </row>
     <row r="31">
@@ -1120,22 +1120,22 @@
         <v>29</v>
       </c>
       <c r="B31" t="n">
-        <v>0</v>
+        <v>174</v>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>2710.069390243903</v>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>1432.176609756098</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>-514.0203738682926</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>38.20672403060977</v>
       </c>
     </row>
     <row r="32">
@@ -1143,22 +1143,22 @@
         <v>30</v>
       </c>
       <c r="B32" t="n">
-        <v>0</v>
+        <v>178</v>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>2507.392</v>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>209.083</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>-433.724315</v>
       </c>
       <c r="G32" t="n">
-        <v>0</v>
+        <v>64.47139527499999</v>
       </c>
     </row>
     <row r="33">
@@ -1166,22 +1166,22 @@
         <v>31</v>
       </c>
       <c r="B33" t="n">
-        <v>0</v>
+        <v>184</v>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>4772.642142857143</v>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>188.1504285714286</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>-424.7477523428572</v>
       </c>
       <c r="G33" t="n">
-        <v>0</v>
+        <v>128.2795580371429</v>
       </c>
     </row>
     <row r="34">
@@ -1189,22 +1189,22 @@
         <v>32</v>
       </c>
       <c r="B34" t="n">
-        <v>0</v>
+        <v>186</v>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>3988.456560975611</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>94.82302439024383</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>0</v>
+        <v>-419.1945213853659</v>
       </c>
       <c r="G34" t="n">
-        <v>0</v>
+        <v>110.7612683232927</v>
       </c>
     </row>
     <row r="35">
@@ -1212,22 +1212,22 @@
         <v>33</v>
       </c>
       <c r="B35" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="C35" t="n">
-        <v>0</v>
+        <v>1547.499904761905</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>1899.487</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>-537.9672175999999</v>
       </c>
       <c r="G35" t="n">
-        <v>0</v>
+        <v>-12.82912067595238</v>
       </c>
     </row>
     <row r="36">
@@ -1235,22 +1235,22 @@
         <v>34</v>
       </c>
       <c r="B36" t="n">
-        <v>0</v>
+        <v>193</v>
       </c>
       <c r="C36" t="n">
-        <v>0</v>
+        <v>819.9459999999999</v>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>2248.5385</v>
       </c>
       <c r="E36" t="n">
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>-579.7087913</v>
       </c>
       <c r="G36" t="n">
-        <v>0</v>
+        <v>-41.08562164</v>
       </c>
     </row>
     <row r="37">
@@ -1258,22 +1258,22 @@
         <v>35</v>
       </c>
       <c r="B37" t="n">
-        <v>0</v>
+        <v>194</v>
       </c>
       <c r="C37" t="n">
-        <v>0</v>
+        <v>2880.965999999999</v>
       </c>
       <c r="D37" t="n">
-        <v>0</v>
+        <v>1851.914</v>
       </c>
       <c r="E37" t="n">
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>0</v>
+        <v>-557.2285552000001</v>
       </c>
       <c r="G37" t="n">
-        <v>0</v>
+        <v>24.38440803499999</v>
       </c>
     </row>
     <row r="38">
@@ -1281,22 +1281,22 @@
         <v>36</v>
       </c>
       <c r="B38" t="n">
-        <v>0</v>
+        <v>196</v>
       </c>
       <c r="C38" t="n">
-        <v>0</v>
+        <v>1925.654</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>2046.721</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>-540.5400364</v>
       </c>
       <c r="G38" t="n">
-        <v>0</v>
+        <v>-4.328580429999999</v>
       </c>
     </row>
     <row r="39">
@@ -1304,22 +1304,22 @@
         <v>37</v>
       </c>
       <c r="B39" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>6264.645999999999</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>22.97800000000001</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>0</v>
+        <v>-406.7351942857143</v>
       </c>
       <c r="G39" t="n">
-        <v>0</v>
+        <v>176.0832530657142</v>
       </c>
     </row>
     <row r="40">
@@ -1327,22 +1327,22 @@
         <v>38</v>
       </c>
       <c r="B40" t="n">
-        <v>0</v>
+        <v>202</v>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>5196.214571428571</v>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>250.9124285714286</v>
       </c>
       <c r="E40" t="n">
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>0</v>
+        <v>-422.2622887714285</v>
       </c>
       <c r="G40" t="n">
-        <v>0</v>
+        <v>138.6949383392857</v>
       </c>
     </row>
     <row r="41">
@@ -1350,22 +1350,22 @@
         <v>39</v>
       </c>
       <c r="B41" t="n">
-        <v>0</v>
+        <v>204</v>
       </c>
       <c r="C41" t="n">
-        <v>0</v>
+        <v>2378.426303797468</v>
       </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>254.0398481012658</v>
       </c>
       <c r="E41" t="n">
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>0</v>
+        <v>-430.3695803797468</v>
       </c>
       <c r="G41" t="n">
-        <v>0</v>
+        <v>60.37606567335443</v>
       </c>
     </row>
     <row r="42">
@@ -1373,22 +1373,22 @@
         <v>40</v>
       </c>
       <c r="B42" t="n">
-        <v>0</v>
+        <v>206</v>
       </c>
       <c r="C42" t="n">
-        <v>0</v>
+        <v>1605.421210526316</v>
       </c>
       <c r="D42" t="n">
-        <v>0</v>
+        <v>2253.286578947368</v>
       </c>
       <c r="E42" t="n">
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>0</v>
+        <v>-571.4939884315789</v>
       </c>
       <c r="G42" t="n">
-        <v>0</v>
+        <v>-17.30791489894735</v>
       </c>
     </row>
     <row r="43">
@@ -1396,22 +1396,22 @@
         <v>41</v>
       </c>
       <c r="B43" t="n">
-        <v>0</v>
+        <v>208</v>
       </c>
       <c r="C43" t="n">
-        <v>0</v>
+        <v>3317.312333333333</v>
       </c>
       <c r="D43" t="n">
-        <v>0</v>
+        <v>624.0768333333333</v>
       </c>
       <c r="E43" t="n">
         <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>0</v>
+        <v>-441.5062237333333</v>
       </c>
       <c r="G43" t="n">
-        <v>0</v>
+        <v>76.12594108166667</v>
       </c>
     </row>
     <row r="44">
@@ -1419,22 +1419,22 @@
         <v>42</v>
       </c>
       <c r="B44" t="n">
-        <v>0</v>
+        <v>209</v>
       </c>
       <c r="C44" t="n">
-        <v>0</v>
+        <v>1641.35</v>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>1212.77</v>
       </c>
       <c r="E44" t="n">
         <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>0</v>
+        <v>-498.8534022</v>
       </c>
       <c r="G44" t="n">
-        <v>0</v>
+        <v>9.600669304999997</v>
       </c>
     </row>
     <row r="45">
@@ -1442,22 +1442,22 @@
         <v>43</v>
       </c>
       <c r="B45" t="n">
-        <v>0</v>
+        <v>210</v>
       </c>
       <c r="C45" t="n">
-        <v>0</v>
+        <v>3276.012000000001</v>
       </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>921.3943846153846</v>
       </c>
       <c r="E45" t="n">
         <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>0</v>
+        <v>-454.5324691384615</v>
       </c>
       <c r="G45" t="n">
-        <v>0</v>
+        <v>66.13665327461538</v>
       </c>
     </row>
     <row r="46">
@@ -1465,22 +1465,22 @@
         <v>44</v>
       </c>
       <c r="B46" t="n">
-        <v>0</v>
+        <v>212</v>
       </c>
       <c r="C46" t="n">
-        <v>0</v>
+        <v>918.9178571428571</v>
       </c>
       <c r="D46" t="n">
-        <v>0</v>
+        <v>2746.892285714286</v>
       </c>
       <c r="E46" t="n">
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>0</v>
+        <v>-593.2906712285715</v>
       </c>
       <c r="G46" t="n">
-        <v>0</v>
+        <v>-53.25975977785715</v>
       </c>
     </row>
     <row r="47">
@@ -1488,22 +1488,22 @@
         <v>45</v>
       </c>
       <c r="B47" t="n">
-        <v>0</v>
+        <v>215</v>
       </c>
       <c r="C47" t="n">
-        <v>0</v>
+        <v>2999.937</v>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>3321.793</v>
       </c>
       <c r="E47" t="n">
         <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>0</v>
+        <v>-611.4916962</v>
       </c>
       <c r="G47" t="n">
-        <v>0</v>
+        <v>-10.79646967000001</v>
       </c>
     </row>
     <row r="48">
@@ -1511,22 +1511,22 @@
         <v>46</v>
       </c>
       <c r="B48" t="n">
-        <v>0</v>
+        <v>217</v>
       </c>
       <c r="C48" t="n">
-        <v>0</v>
+        <v>1455.255909090909</v>
       </c>
       <c r="D48" t="n">
-        <v>0</v>
+        <v>1971.038727272728</v>
       </c>
       <c r="E48" t="n">
         <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>0</v>
+        <v>-561.7020352181819</v>
       </c>
       <c r="G48" t="n">
-        <v>0</v>
+        <v>-17.85524053227274</v>
       </c>
     </row>
     <row r="49">
@@ -1534,22 +1534,22 @@
         <v>47</v>
       </c>
       <c r="B49" t="n">
-        <v>0</v>
+        <v>219</v>
       </c>
       <c r="C49" t="n">
-        <v>0</v>
+        <v>4072.716414634147</v>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>108.1661463414634</v>
       </c>
       <c r="E49" t="n">
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>0</v>
+        <v>-421.7709270439025</v>
       </c>
       <c r="G49" t="n">
-        <v>0</v>
+        <v>109.73381976</v>
       </c>
     </row>
     <row r="50">
@@ -1557,22 +1557,22 @@
         <v>48</v>
       </c>
       <c r="B50" t="n">
-        <v>0</v>
+        <v>223</v>
       </c>
       <c r="C50" t="n">
-        <v>0</v>
+        <v>3195.234705882353</v>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>1057.362</v>
       </c>
       <c r="E50" t="n">
         <v>0</v>
       </c>
       <c r="F50" t="n">
-        <v>0</v>
+        <v>-492.8028849764706</v>
       </c>
       <c r="G50" t="n">
-        <v>0</v>
+        <v>57.07734277382354</v>
       </c>
     </row>
     <row r="51">
@@ -1580,22 +1580,22 @@
         <v>49</v>
       </c>
       <c r="B51" t="n">
-        <v>0</v>
+        <v>225</v>
       </c>
       <c r="C51" t="n">
-        <v>0</v>
+        <v>1694.502727272727</v>
       </c>
       <c r="D51" t="n">
-        <v>0</v>
+        <v>1591.010545454546</v>
       </c>
       <c r="E51" t="n">
         <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>0</v>
+        <v>-524.0009958909091</v>
       </c>
       <c r="G51" t="n">
-        <v>0</v>
+        <v>-1.064879741818196</v>
       </c>
     </row>
     <row r="52">
@@ -1603,22 +1603,22 @@
         <v>50</v>
       </c>
       <c r="B52" t="n">
-        <v>0</v>
+        <v>226</v>
       </c>
       <c r="C52" t="n">
-        <v>0</v>
+        <v>3530.118838709676</v>
       </c>
       <c r="D52" t="n">
-        <v>0</v>
+        <v>468.1675483870969</v>
       </c>
       <c r="E52" t="n">
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>0</v>
+        <v>-450.0953327354839</v>
       </c>
       <c r="G52" t="n">
-        <v>0</v>
+        <v>84.14871068532253</v>
       </c>
     </row>
     <row r="53">
@@ -1626,22 +1626,22 @@
         <v>51</v>
       </c>
       <c r="B53" t="n">
-        <v>0</v>
+        <v>227</v>
       </c>
       <c r="C53" t="n">
-        <v>0</v>
+        <v>3184.218</v>
       </c>
       <c r="D53" t="n">
-        <v>0</v>
+        <v>621.865</v>
       </c>
       <c r="E53" t="n">
         <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>0</v>
+        <v>-451.6743032</v>
       </c>
       <c r="G53" t="n">
-        <v>0</v>
+        <v>70.89208870499999</v>
       </c>
     </row>
     <row r="54">
@@ -1649,22 +1649,22 @@
         <v>52</v>
       </c>
       <c r="B54" t="n">
-        <v>0</v>
+        <v>232</v>
       </c>
       <c r="C54" t="n">
-        <v>0</v>
+        <v>401.311636363636</v>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>3961.982636363636</v>
       </c>
       <c r="E54" t="n">
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>0</v>
+        <v>-656.7345793090909</v>
       </c>
       <c r="G54" t="n">
-        <v>0</v>
+        <v>-107.0713108604546</v>
       </c>
     </row>
     <row r="55">
@@ -1672,22 +1672,22 @@
         <v>53</v>
       </c>
       <c r="B55" t="n">
-        <v>0</v>
+        <v>235</v>
       </c>
       <c r="C55" t="n">
-        <v>0</v>
+        <v>4079.419</v>
       </c>
       <c r="D55" t="n">
-        <v>0</v>
+        <v>411.496</v>
       </c>
       <c r="E55" t="n">
         <v>0</v>
       </c>
       <c r="F55" t="n">
-        <v>0</v>
+        <v>-451.0743954</v>
       </c>
       <c r="G55" t="n">
-        <v>0</v>
+        <v>102.51237108</v>
       </c>
     </row>
     <row r="56">
@@ -1695,22 +1695,22 @@
         <v>54</v>
       </c>
       <c r="B56" t="n">
-        <v>0</v>
+        <v>239</v>
       </c>
       <c r="C56" t="n">
-        <v>0</v>
+        <v>3498.536999999999</v>
       </c>
       <c r="D56" t="n">
-        <v>0</v>
+        <v>549.021</v>
       </c>
       <c r="E56" t="n">
         <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>0</v>
+        <v>-436.1584134</v>
       </c>
       <c r="G56" t="n">
-        <v>0</v>
+        <v>85.091795495</v>
       </c>
     </row>
     <row r="57">
@@ -1718,22 +1718,22 @@
         <v>55</v>
       </c>
       <c r="B57" t="n">
-        <v>0</v>
+        <v>241</v>
       </c>
       <c r="C57" t="n">
-        <v>0</v>
+        <v>5229.318</v>
       </c>
       <c r="D57" t="n">
-        <v>0</v>
+        <v>280.252</v>
       </c>
       <c r="E57" t="n">
         <v>0</v>
       </c>
       <c r="F57" t="n">
-        <v>0</v>
+        <v>-412.897455</v>
       </c>
       <c r="G57" t="n">
-        <v>0</v>
+        <v>136.36770352</v>
       </c>
     </row>
     <row r="58">
@@ -1741,22 +1741,22 @@
         <v>56</v>
       </c>
       <c r="B58" t="n">
-        <v>0</v>
+        <v>243</v>
       </c>
       <c r="C58" t="n">
-        <v>0</v>
+        <v>1335.945935483871</v>
       </c>
       <c r="D58" t="n">
-        <v>0</v>
+        <v>1885.720967741936</v>
       </c>
       <c r="E58" t="n">
         <v>0</v>
       </c>
       <c r="F58" t="n">
-        <v>0</v>
+        <v>-556.5021458193548</v>
       </c>
       <c r="G58" t="n">
-        <v>0</v>
+        <v>-16.26478529435485</v>
       </c>
     </row>
     <row r="59">
@@ -1764,22 +1764,22 @@
         <v>57</v>
       </c>
       <c r="B59" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C59" t="n">
-        <v>0</v>
+        <v>4852.394571428572</v>
       </c>
       <c r="D59" t="n">
-        <v>0</v>
+        <v>194.2727142857142</v>
       </c>
       <c r="E59" t="n">
         <v>0</v>
       </c>
       <c r="F59" t="n">
-        <v>0</v>
+        <v>-425.1530031428571</v>
       </c>
       <c r="G59" t="n">
-        <v>0</v>
+        <v>130.2751602378572</v>
       </c>
     </row>
     <row r="60">
@@ -1787,22 +1787,22 @@
         <v>58</v>
       </c>
       <c r="B60" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="C60" t="n">
-        <v>0</v>
+        <v>870.8624285714285</v>
       </c>
       <c r="D60" t="n">
-        <v>0</v>
+        <v>3043.383285714286</v>
       </c>
       <c r="E60" t="n">
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>0</v>
+        <v>-631.4983085714285</v>
       </c>
       <c r="G60" t="n">
-        <v>0</v>
+        <v>-62.00590391642859</v>
       </c>
     </row>
     <row r="61">
@@ -1810,22 +1810,22 @@
         <v>59</v>
       </c>
       <c r="B61" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="C61" t="n">
-        <v>0</v>
+        <v>2206.937</v>
       </c>
       <c r="D61" t="n">
-        <v>0</v>
+        <v>967.162</v>
       </c>
       <c r="E61" t="n">
         <v>0</v>
       </c>
       <c r="F61" t="n">
-        <v>0</v>
+        <v>-470.8646932</v>
       </c>
       <c r="G61" t="n">
-        <v>0</v>
+        <v>34.39400462</v>
       </c>
     </row>
     <row r="62">
@@ -1833,22 +1833,22 @@
         <v>60</v>
       </c>
       <c r="B62" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C62" t="n">
-        <v>0</v>
+        <v>2962.368714285713</v>
       </c>
       <c r="D62" t="n">
-        <v>0</v>
+        <v>689.4412857142859</v>
       </c>
       <c r="E62" t="n">
         <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>0</v>
+        <v>-440.9629365142857</v>
       </c>
       <c r="G62" t="n">
-        <v>0</v>
+        <v>63.82182995499997</v>
       </c>
     </row>
     <row r="63">
@@ -1856,22 +1856,22 @@
         <v>61</v>
       </c>
       <c r="B63" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="C63" t="n">
-        <v>0</v>
+        <v>1357.127333333333</v>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>2027.260333333333</v>
       </c>
       <c r="E63" t="n">
         <v>0</v>
       </c>
       <c r="F63" t="n">
-        <v>0</v>
+        <v>-573.6512277333334</v>
       </c>
       <c r="G63" t="n">
-        <v>0</v>
+        <v>-24.33612080166667</v>
       </c>
     </row>
     <row r="64">
@@ -1879,22 +1879,22 @@
         <v>62</v>
       </c>
       <c r="B64" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="C64" t="n">
-        <v>0</v>
+        <v>1591.107206896552</v>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>889.9376551724138</v>
       </c>
       <c r="E64" t="n">
         <v>0</v>
       </c>
       <c r="F64" t="n">
-        <v>0</v>
+        <v>-496.9183250965517</v>
       </c>
       <c r="G64" t="n">
-        <v>0</v>
+        <v>18.78396745603448</v>
       </c>
     </row>
     <row r="65">
@@ -1902,22 +1902,22 @@
         <v>63</v>
       </c>
       <c r="B65" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="C65" t="n">
-        <v>0</v>
+        <v>3942.198</v>
       </c>
       <c r="D65" t="n">
-        <v>0</v>
+        <v>276.543</v>
       </c>
       <c r="E65" t="n">
         <v>0</v>
       </c>
       <c r="F65" t="n">
-        <v>0</v>
+        <v>-426.4654854</v>
       </c>
       <c r="G65" t="n">
-        <v>0</v>
+        <v>102.64023768</v>
       </c>
     </row>
     <row r="66">
@@ -1925,22 +1925,22 @@
         <v>64</v>
       </c>
       <c r="B66" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="C66" t="n">
-        <v>0</v>
+        <v>2606.615741935484</v>
       </c>
       <c r="D66" t="n">
-        <v>0</v>
+        <v>909.3630000000003</v>
       </c>
       <c r="E66" t="n">
         <v>0</v>
       </c>
       <c r="F66" t="n">
-        <v>0</v>
+        <v>-484.8810560064516</v>
       </c>
       <c r="G66" t="n">
-        <v>0</v>
+        <v>46.60549129419353</v>
       </c>
     </row>
     <row r="67">
@@ -1948,22 +1948,22 @@
         <v>65</v>
       </c>
       <c r="B67" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="C67" t="n">
-        <v>0</v>
+        <v>2477.931</v>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>1178.769</v>
       </c>
       <c r="E67" t="n">
         <v>0</v>
       </c>
       <c r="F67" t="n">
-        <v>0</v>
+        <v>-488.3328728</v>
       </c>
       <c r="G67" t="n">
-        <v>0</v>
+        <v>35.95414214</v>
       </c>
     </row>
     <row r="68">
@@ -1971,22 +1971,22 @@
         <v>66</v>
       </c>
       <c r="B68" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="C68" t="n">
-        <v>0</v>
+        <v>2093.914317073171</v>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>1170.893170731707</v>
       </c>
       <c r="E68" t="n">
         <v>0</v>
       </c>
       <c r="F68" t="n">
-        <v>0</v>
+        <v>-520.034615204878</v>
       </c>
       <c r="G68" t="n">
-        <v>0</v>
+        <v>20.36819213487807</v>
       </c>
     </row>
     <row r="69">
@@ -1994,22 +1994,22 @@
         <v>67</v>
       </c>
       <c r="B69" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="C69" t="n">
-        <v>0</v>
+        <v>91.1818571428571</v>
       </c>
       <c r="D69" t="n">
-        <v>0</v>
+        <v>5089.029714285714</v>
       </c>
       <c r="E69" t="n">
         <v>0</v>
       </c>
       <c r="F69" t="n">
-        <v>0</v>
+        <v>-743.0059369142857</v>
       </c>
       <c r="G69" t="n">
-        <v>0</v>
+        <v>-141.1689260835714</v>
       </c>
     </row>
     <row r="70">
@@ -2017,22 +2017,22 @@
         <v>68</v>
       </c>
       <c r="B70" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="C70" t="n">
-        <v>0</v>
+        <v>2588.705142857143</v>
       </c>
       <c r="D70" t="n">
-        <v>0</v>
+        <v>1413.355</v>
       </c>
       <c r="E70" t="n">
         <v>0</v>
       </c>
       <c r="F70" t="n">
-        <v>0</v>
+        <v>-519.8093698571429</v>
       </c>
       <c r="G70" t="n">
-        <v>0</v>
+        <v>34.10906637642859</v>
       </c>
     </row>
     <row r="71">
@@ -2040,22 +2040,22 @@
         <v>69</v>
       </c>
       <c r="B71" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="C71" t="n">
-        <v>0</v>
+        <v>1414.799</v>
       </c>
       <c r="D71" t="n">
-        <v>0</v>
+        <v>1383.522</v>
       </c>
       <c r="E71" t="n">
         <v>0</v>
       </c>
       <c r="F71" t="n">
-        <v>0</v>
+        <v>-516.3954851999999</v>
       </c>
       <c r="G71" t="n">
-        <v>0</v>
+        <v>0.06237605499999788</v>
       </c>
     </row>
     <row r="72">
@@ -2063,22 +2063,22 @@
         <v>70</v>
       </c>
       <c r="B72" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="C72" t="n">
-        <v>0</v>
+        <v>1696.832</v>
       </c>
       <c r="D72" t="n">
-        <v>0</v>
+        <v>2374.626</v>
       </c>
       <c r="E72" t="n">
         <v>0</v>
       </c>
       <c r="F72" t="n">
-        <v>0</v>
+        <v>-555.9352269999999</v>
       </c>
       <c r="G72" t="n">
-        <v>0</v>
+        <v>-21.80704658000001</v>
       </c>
     </row>
     <row r="73">
@@ -2086,22 +2086,22 @@
         <v>71</v>
       </c>
       <c r="B73" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="C73" t="n">
-        <v>0</v>
+        <v>3501.190750000002</v>
       </c>
       <c r="D73" t="n">
-        <v>0</v>
+        <v>485.0264999999998</v>
       </c>
       <c r="E73" t="n">
         <v>0</v>
       </c>
       <c r="F73" t="n">
-        <v>0</v>
+        <v>-443.56600405</v>
       </c>
       <c r="G73" t="n">
-        <v>0</v>
+        <v>83.85038975125003</v>
       </c>
     </row>
     <row r="74">
@@ -2109,22 +2109,22 @@
         <v>72</v>
       </c>
       <c r="B74" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="C74" t="n">
-        <v>0</v>
+        <v>1895.772</v>
       </c>
       <c r="D74" t="n">
-        <v>0</v>
+        <v>507.5399999999998</v>
       </c>
       <c r="E74" t="n">
         <v>0</v>
       </c>
       <c r="F74" t="n">
-        <v>0</v>
+        <v>-451.8054646</v>
       </c>
       <c r="G74" t="n">
-        <v>0</v>
+        <v>39.74268578000002</v>
       </c>
     </row>
     <row r="75">
@@ -2132,22 +2132,22 @@
         <v>73</v>
       </c>
       <c r="B75" t="n">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="C75" t="n">
-        <v>0</v>
+        <v>1002.092</v>
       </c>
       <c r="D75" t="n">
-        <v>0</v>
+        <v>1063.13587804878</v>
       </c>
       <c r="E75" t="n">
         <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>0</v>
+        <v>-491.3775999463414</v>
       </c>
       <c r="G75" t="n">
-        <v>0</v>
+        <v>-0.4341953863414467</v>
       </c>
     </row>
     <row r="76">
@@ -2155,22 +2155,22 @@
         <v>74</v>
       </c>
       <c r="B76" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="C76" t="n">
-        <v>0</v>
+        <v>495.6949999999999</v>
       </c>
       <c r="D76" t="n">
-        <v>0</v>
+        <v>2860.151</v>
       </c>
       <c r="E76" t="n">
         <v>0</v>
       </c>
       <c r="F76" t="n">
-        <v>0</v>
+        <v>-603.2055792</v>
       </c>
       <c r="G76" t="n">
-        <v>0</v>
+        <v>-64.82355931000001</v>
       </c>
     </row>
     <row r="77">
@@ -2178,22 +2178,22 @@
         <v>75</v>
       </c>
       <c r="B77" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="C77" t="n">
-        <v>0</v>
+        <v>1157.077</v>
       </c>
       <c r="D77" t="n">
-        <v>0</v>
+        <v>1518.949</v>
       </c>
       <c r="E77" t="n">
         <v>0</v>
       </c>
       <c r="F77" t="n">
-        <v>0</v>
+        <v>-508.564791</v>
       </c>
       <c r="G77" t="n">
-        <v>0</v>
+        <v>-12.09595504</v>
       </c>
     </row>
     <row r="78">
@@ -2201,22 +2201,22 @@
         <v>76</v>
       </c>
       <c r="B78" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="C78" t="n">
-        <v>0</v>
+        <v>3859.607</v>
       </c>
       <c r="D78" t="n">
-        <v>0</v>
+        <v>272.3800000000001</v>
       </c>
       <c r="E78" t="n">
         <v>0</v>
       </c>
       <c r="F78" t="n">
-        <v>0</v>
+        <v>-428.8861056</v>
       </c>
       <c r="G78" t="n">
-        <v>0</v>
+        <v>101.303990485</v>
       </c>
     </row>
     <row r="79">
@@ -2224,22 +2224,22 @@
         <v>77</v>
       </c>
       <c r="B79" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="C79" t="n">
-        <v>0</v>
+        <v>1098.2075</v>
       </c>
       <c r="D79" t="n">
-        <v>0</v>
+        <v>1920.89725</v>
       </c>
       <c r="E79" t="n">
         <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>0</v>
+        <v>-542.5019605</v>
       </c>
       <c r="G79" t="n">
-        <v>0</v>
+        <v>-20.2834454175</v>
       </c>
     </row>
     <row r="80">
@@ -2247,22 +2247,22 @@
         <v>78</v>
       </c>
       <c r="B80" t="n">
-        <v>0</v>
+        <v>77</v>
       </c>
       <c r="C80" t="n">
-        <v>0</v>
+        <v>4007.409365853659</v>
       </c>
       <c r="D80" t="n">
-        <v>0</v>
+        <v>504.2338780487804</v>
       </c>
       <c r="E80" t="n">
         <v>0</v>
       </c>
       <c r="F80" t="n">
-        <v>0</v>
+        <v>-447.0940627560976</v>
       </c>
       <c r="G80" t="n">
-        <v>0</v>
+        <v>98.12219584439029</v>
       </c>
     </row>
     <row r="81">
@@ -2270,22 +2270,22 @@
         <v>79</v>
       </c>
       <c r="B81" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="C81" t="n">
-        <v>0</v>
+        <v>2306.852467532468</v>
       </c>
       <c r="D81" t="n">
-        <v>0</v>
+        <v>338.7829090909092</v>
       </c>
       <c r="E81" t="n">
         <v>0</v>
       </c>
       <c r="F81" t="n">
-        <v>0</v>
+        <v>-436.4776856727273</v>
       </c>
       <c r="G81" t="n">
-        <v>0</v>
+        <v>55.86668966253249</v>
       </c>
     </row>
     <row r="82">
@@ -2293,22 +2293,22 @@
         <v>80</v>
       </c>
       <c r="B82" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="C82" t="n">
-        <v>0</v>
+        <v>370.4155714285716</v>
       </c>
       <c r="D82" t="n">
-        <v>0</v>
+        <v>3324.260571428571</v>
       </c>
       <c r="E82" t="n">
         <v>0</v>
       </c>
       <c r="F82" t="n">
-        <v>0</v>
+        <v>-617.3596889714286</v>
       </c>
       <c r="G82" t="n">
-        <v>0</v>
+        <v>-81.42250351928571</v>
       </c>
     </row>
     <row r="83">
@@ -2316,22 +2316,22 @@
         <v>81</v>
       </c>
       <c r="B83" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="C83" t="n">
-        <v>0</v>
+        <v>5162.089</v>
       </c>
       <c r="D83" t="n">
-        <v>0</v>
+        <v>4.367</v>
       </c>
       <c r="E83" t="n">
         <v>0</v>
       </c>
       <c r="F83" t="n">
-        <v>0</v>
+        <v>-411.33786</v>
       </c>
       <c r="G83" t="n">
-        <v>0</v>
+        <v>145.649312225</v>
       </c>
     </row>
     <row r="84">
@@ -2339,22 +2339,22 @@
         <v>82</v>
       </c>
       <c r="B84" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="C84" t="n">
-        <v>0</v>
+        <v>6481.944333333333</v>
       </c>
       <c r="D84" t="n">
-        <v>0</v>
+        <v>17.032</v>
       </c>
       <c r="E84" t="n">
         <v>0</v>
       </c>
       <c r="F84" t="n">
-        <v>0</v>
+        <v>-410.1599055333333</v>
       </c>
       <c r="G84" t="n">
-        <v>0</v>
+        <v>181.690864375</v>
       </c>
     </row>
     <row r="85">
@@ -2362,22 +2362,22 @@
         <v>83</v>
       </c>
       <c r="B85" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="C85" t="n">
-        <v>0</v>
+        <v>1096.135714285714</v>
       </c>
       <c r="D85" t="n">
-        <v>0</v>
+        <v>2865.592</v>
       </c>
       <c r="E85" t="n">
         <v>0</v>
       </c>
       <c r="F85" t="n">
-        <v>0</v>
+        <v>-588.6831728571428</v>
       </c>
       <c r="G85" t="n">
-        <v>0</v>
+        <v>-47.28097123285714</v>
       </c>
     </row>
     <row r="86">
@@ -2385,22 +2385,22 @@
         <v>84</v>
       </c>
       <c r="B86" t="n">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="C86" t="n">
-        <v>0</v>
+        <v>310.5940000000001</v>
       </c>
       <c r="D86" t="n">
-        <v>0</v>
+        <v>8236.696</v>
       </c>
       <c r="E86" t="n">
         <v>0</v>
       </c>
       <c r="F86" t="n">
-        <v>0</v>
+        <v>-1080.825698</v>
       </c>
       <c r="G86" t="n">
-        <v>0</v>
+        <v>-245.3728373</v>
       </c>
     </row>
     <row r="87">
@@ -2408,22 +2408,22 @@
         <v>85</v>
       </c>
       <c r="B87" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="C87" t="n">
-        <v>0</v>
+        <v>416.1759999999999</v>
       </c>
       <c r="D87" t="n">
-        <v>0</v>
+        <v>1590.875</v>
       </c>
       <c r="E87" t="n">
         <v>0</v>
       </c>
       <c r="F87" t="n">
-        <v>0</v>
+        <v>-511.239003</v>
       </c>
       <c r="G87" t="n">
-        <v>0</v>
+        <v>-33.281449525</v>
       </c>
     </row>
     <row r="88">
@@ -2431,22 +2431,22 @@
         <v>86</v>
       </c>
       <c r="B88" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="C88" t="n">
-        <v>0</v>
+        <v>1547.471</v>
       </c>
       <c r="D88" t="n">
-        <v>0</v>
+        <v>542.495</v>
       </c>
       <c r="E88" t="n">
         <v>0</v>
       </c>
       <c r="F88" t="n">
-        <v>0</v>
+        <v>-448.8756316</v>
       </c>
       <c r="G88" t="n">
-        <v>0</v>
+        <v>27.958334165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>